<commit_message>
fix save/load logic, applied SOLID though not perfect
</commit_message>
<xml_diff>
--- a/books.xlsx
+++ b/books.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>ID</t>
   </si>
@@ -23,10 +23,16 @@
     <t>Author</t>
   </si>
   <si>
-    <t>bomba</t>
+    <t>meow</t>
   </si>
   <si>
-    <t>clat</t>
+    <t>cat</t>
+  </si>
+  <si>
+    <t>woof</t>
+  </si>
+  <si>
+    <t>dawg</t>
   </si>
 </sst>
 </file>
@@ -71,7 +77,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -87,7 +93,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n" s="0">
-        <v>9.0</v>
+        <v>1.0</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>3</v>
@@ -96,6 +102,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>